<commit_message>
Improved Error reporting by reporting all columns that have errors.
</commit_message>
<xml_diff>
--- a/src/test/resources/test-5problems.xlsx
+++ b/src/test/resources/test-5problems.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-20.04\home\tvandenberghe\dev\ears3\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\mephistophilus\MyGitRepositories\ears3\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18CE8D68-A9C4-4FD5-BFA5-C05BBA4CFEA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95FD1550-F68E-4EC1-9AD1-9BD6D4C1066C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="332" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30525" yWindow="1395" windowWidth="21600" windowHeight="11295" tabRatio="332" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3394" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3405" uniqueCount="333">
   <si>
     <t>Date</t>
   </si>
@@ -1458,7 +1458,7 @@
     <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="286">
+  <dxfs count="292">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1491,7 +1491,37 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
       </font>
       <fill>
         <patternFill>
@@ -1531,7 +1561,7 @@
     </dxf>
     <dxf>
       <font>
-        <color auto="1"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
@@ -1595,7 +1625,27 @@
       </font>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1611,6 +1661,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -1671,11 +1731,41 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1691,6 +1781,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -1715,7 +1825,27 @@
       </font>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1751,6 +1881,46 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -1791,11 +1961,31 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1811,6 +2001,36 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -1851,11 +2071,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC000"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1871,6 +2091,16 @@
     </dxf>
     <dxf>
       <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -1905,7 +2135,17 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC000"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1921,11 +2161,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color auto="1"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1941,6 +2191,36 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -1961,11 +2241,21 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC000"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1981,11 +2271,41 @@
     </dxf>
     <dxf>
       <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2001,11 +2321,31 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2021,11 +2361,31 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2041,11 +2401,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2065,6 +2425,16 @@
       </font>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
@@ -2081,11 +2451,41 @@
     </dxf>
     <dxf>
       <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2101,11 +2501,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color auto="1"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2125,7 +2535,37 @@
       </font>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2141,11 +2581,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color auto="1"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2165,6 +2605,16 @@
       </font>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
@@ -2181,7 +2631,27 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
       </font>
       <fill>
         <patternFill>
@@ -2220,6 +2690,33 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <color rgb="FF9C0006"/>
       </font>
@@ -2231,11 +2728,31 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2251,11 +2768,41 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2271,11 +2818,31 @@
     </dxf>
     <dxf>
       <font>
-        <color auto="1"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2291,11 +2858,31 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2311,11 +2898,31 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2331,7 +2938,7 @@
     </dxf>
     <dxf>
       <font>
-        <color auto="1"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
@@ -2381,11 +2988,141 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2401,6 +3138,46 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -2425,6 +3202,36 @@
       </font>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
@@ -2441,11 +3248,61 @@
     </dxf>
     <dxf>
       <font>
-        <color auto="1"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2475,7 +3332,27 @@
       </font>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2501,6 +3378,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -2521,11 +3418,11 @@
     </dxf>
     <dxf>
       <font>
-        <color auto="1"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC000"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2571,11 +3468,11 @@
     </dxf>
     <dxf>
       <font>
-        <color auto="1"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC000"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2591,11 +3488,21 @@
     </dxf>
     <dxf>
       <font>
-        <color auto="1"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC000"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2611,11 +3518,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color auto="1"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2630,9 +3537,32 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
       <fill>
         <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2648,11 +3578,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color auto="1"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2668,11 +3608,31 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color auto="1"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2688,16 +3648,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -2708,7 +3658,27 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
       </font>
       <fill>
         <patternFill>
@@ -2733,916 +3703,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4453,14 +4513,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:L235" totalsRowShown="0" headerRowDxfId="285">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:L235" totalsRowShown="0" headerRowDxfId="291">
   <autoFilter ref="A1:L235" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="12">
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Date" dataDxfId="284"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Date" dataDxfId="290"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Hour (B)"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Subject"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Description" dataDxfId="283"/>
-    <tableColumn id="12" xr3:uid="{789140AF-ECDD-49C9-962D-682F73BF1C2E}" name="Remarks" dataDxfId="282"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Description" dataDxfId="289"/>
+    <tableColumn id="12" xr3:uid="{789140AF-ECDD-49C9-962D-682F73BF1C2E}" name="Remarks" dataDxfId="288"/>
     <tableColumn id="13" xr3:uid="{3A757FBE-B7D5-466D-BCDD-D2583B5EC07D}" name="Dist (nm)"/>
     <tableColumn id="1" xr3:uid="{28FDAEE7-A28A-436E-A60C-751D5EB68D42}" name="Time (u)"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="For"/>
@@ -4474,7 +4534,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{DD5B9AB8-C51C-4ABE-9D23-359CA3F04288}" name="Table134" displayName="Table134" ref="A5:AC240" totalsRowShown="0" headerRowDxfId="281" dataDxfId="280">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{DD5B9AB8-C51C-4ABE-9D23-359CA3F04288}" name="Table134" displayName="Table134" ref="A5:AC240" totalsRowShown="0" headerRowDxfId="287" dataDxfId="286">
   <autoFilter ref="A5:AC240" xr:uid="{00000000-0009-0000-0100-000001000000}">
     <filterColumn colId="6">
       <filters>
@@ -4486,76 +4546,76 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="29">
-    <tableColumn id="2" xr3:uid="{8537F5E4-DE86-4A23-9BFF-DBAF106EE11D}" name="Date" dataDxfId="279" dataCellStyle="Neutral"/>
-    <tableColumn id="3" xr3:uid="{E55E821D-D2E5-4612-845F-A66DA34A7F03}" name="Hour" dataDxfId="278" dataCellStyle="Neutral"/>
-    <tableColumn id="32" xr3:uid="{D419F3C5-DB40-4577-B1D8-535F3937D736}" name="Actor" dataDxfId="277" dataCellStyle="Neutral"/>
-    <tableColumn id="22" xr3:uid="{7F1E5ED8-E912-42D4-8C72-7A21366AA497}" name="eventDefinitionId" dataDxfId="276" dataCellStyle="Neutral"/>
-    <tableColumn id="21" xr3:uid="{C9A1DBB6-16F3-4AF5-95AE-5E4E26D9D28D}" name="Program" dataDxfId="275" dataCellStyle="Neutral"/>
-    <tableColumn id="6" xr3:uid="{0B4F15C3-5A29-48DB-B5DA-B32EDF7E2152}" name="Tool" dataDxfId="274" dataCellStyle="Neutral"/>
-    <tableColumn id="15" xr3:uid="{23EF9D9F-EEAC-4532-8A12-70CA5D97A014}" name="Process" dataDxfId="273" dataCellStyle="Neutral"/>
-    <tableColumn id="14" xr3:uid="{ABB295AF-377B-4EFB-837A-24EB5EC8758E}" name="Action" dataDxfId="272" dataCellStyle="Neutral"/>
-    <tableColumn id="16" xr3:uid="{E485F26A-2BBA-4094-A21E-AE2C86D212F3}" name="Label" dataDxfId="271" dataCellStyle="Neutral"/>
-    <tableColumn id="18" xr3:uid="{052671CD-3112-4770-9E57-584DAC75EE42}" name="Station" dataDxfId="270" dataCellStyle="Neutral"/>
-    <tableColumn id="17" xr3:uid="{E60C43AC-26A5-4D77-8163-238B5D43865C}" name="Description" dataDxfId="269" dataCellStyle="Neutral"/>
-    <tableColumn id="31" xr3:uid="{FCEA5263-578B-40A4-A74C-55573412C3AA}" name="Remarks" dataDxfId="268" dataCellStyle="Neutral"/>
-    <tableColumn id="27" xr3:uid="{92059A6A-2B36-4051-9543-5C5758E39437}" name="Dist" dataDxfId="267" dataCellStyle="Neutral"/>
-    <tableColumn id="26" xr3:uid="{C4BF088D-BC48-48BF-BB20-01F7F32163CE}" name="Time" dataDxfId="266" dataCellStyle="Neutral"/>
-    <tableColumn id="24" xr3:uid="{1DE966F9-FCAA-4A5F-9155-2EF97E0F522F}" name="Status" dataDxfId="265" dataCellStyle="Neutral"/>
-    <tableColumn id="29" xr3:uid="{87F59992-94B6-4570-BC85-599C6C120457}" name="Region" dataDxfId="264" dataCellStyle="Neutral"/>
-    <tableColumn id="28" xr3:uid="{6F943A9E-8917-4D9E-B9E7-F4A05FFB81D2}" name="Weather" dataDxfId="263" dataCellStyle="Neutral"/>
-    <tableColumn id="23" xr3:uid="{7894930C-23CD-4521-B98E-3B5BF35910A6}" name="Navigation" dataDxfId="262" dataCellStyle="Neutral"/>
-    <tableColumn id="4" xr3:uid="{1DF1C017-7D5C-4049-8DAB-6EFD6982A8D3}" name="Subject" dataDxfId="261"/>
-    <tableColumn id="5" xr3:uid="{5DC19A03-7D17-498B-872C-75D3C0B8FE97}" name="Description2" dataDxfId="260"/>
-    <tableColumn id="12" xr3:uid="{D1D2B78A-7689-453A-BB50-F1E3BA54F82F}" name="Remarks2" dataDxfId="259"/>
-    <tableColumn id="13" xr3:uid="{46A53FFB-D8FC-4762-A453-F18649266844}" name="Dist (nm)2" dataDxfId="258"/>
-    <tableColumn id="1" xr3:uid="{C4E9AC53-131F-4965-A278-C8805116FF72}" name="Time (u)3" dataDxfId="257"/>
-    <tableColumn id="7" xr3:uid="{CEA136EA-E892-418E-9B76-70DF71C227ED}" name="For4" dataDxfId="256"/>
-    <tableColumn id="8" xr3:uid="{E94A949A-C095-4435-BA47-1E19F13C2CD4}" name="Status5" dataDxfId="255"/>
-    <tableColumn id="9" xr3:uid="{A2004532-A635-4B73-95B0-9A57606A659F}" name="Region6" dataDxfId="254"/>
-    <tableColumn id="10" xr3:uid="{376C73C8-27F3-4D13-8CA3-86B26B6BEABA}" name="Weather7" dataDxfId="253"/>
-    <tableColumn id="11" xr3:uid="{796A7359-26E1-48C4-8A7B-F2AF2A8C071A}" name="Navigation8" dataDxfId="252"/>
-    <tableColumn id="20" xr3:uid="{6CEBCB9B-E078-4B16-BDDF-BCE0F9BE3FE0}" name="original order" dataDxfId="251"/>
+    <tableColumn id="2" xr3:uid="{8537F5E4-DE86-4A23-9BFF-DBAF106EE11D}" name="Date" dataDxfId="285" dataCellStyle="Neutral"/>
+    <tableColumn id="3" xr3:uid="{E55E821D-D2E5-4612-845F-A66DA34A7F03}" name="Hour" dataDxfId="284" dataCellStyle="Neutral"/>
+    <tableColumn id="32" xr3:uid="{D419F3C5-DB40-4577-B1D8-535F3937D736}" name="Actor" dataDxfId="283" dataCellStyle="Neutral"/>
+    <tableColumn id="22" xr3:uid="{7F1E5ED8-E912-42D4-8C72-7A21366AA497}" name="eventDefinitionId" dataDxfId="282" dataCellStyle="Neutral"/>
+    <tableColumn id="21" xr3:uid="{C9A1DBB6-16F3-4AF5-95AE-5E4E26D9D28D}" name="Program" dataDxfId="281" dataCellStyle="Neutral"/>
+    <tableColumn id="6" xr3:uid="{0B4F15C3-5A29-48DB-B5DA-B32EDF7E2152}" name="Tool" dataDxfId="280" dataCellStyle="Neutral"/>
+    <tableColumn id="15" xr3:uid="{23EF9D9F-EEAC-4532-8A12-70CA5D97A014}" name="Process" dataDxfId="279" dataCellStyle="Neutral"/>
+    <tableColumn id="14" xr3:uid="{ABB295AF-377B-4EFB-837A-24EB5EC8758E}" name="Action" dataDxfId="278" dataCellStyle="Neutral"/>
+    <tableColumn id="16" xr3:uid="{E485F26A-2BBA-4094-A21E-AE2C86D212F3}" name="Label" dataDxfId="277" dataCellStyle="Neutral"/>
+    <tableColumn id="18" xr3:uid="{052671CD-3112-4770-9E57-584DAC75EE42}" name="Station" dataDxfId="276" dataCellStyle="Neutral"/>
+    <tableColumn id="17" xr3:uid="{E60C43AC-26A5-4D77-8163-238B5D43865C}" name="Description" dataDxfId="275" dataCellStyle="Neutral"/>
+    <tableColumn id="31" xr3:uid="{FCEA5263-578B-40A4-A74C-55573412C3AA}" name="Remarks" dataDxfId="274" dataCellStyle="Neutral"/>
+    <tableColumn id="27" xr3:uid="{92059A6A-2B36-4051-9543-5C5758E39437}" name="Dist" dataDxfId="273" dataCellStyle="Neutral"/>
+    <tableColumn id="26" xr3:uid="{C4BF088D-BC48-48BF-BB20-01F7F32163CE}" name="Time" dataDxfId="272" dataCellStyle="Neutral"/>
+    <tableColumn id="24" xr3:uid="{1DE966F9-FCAA-4A5F-9155-2EF97E0F522F}" name="Status" dataDxfId="271" dataCellStyle="Neutral"/>
+    <tableColumn id="29" xr3:uid="{87F59992-94B6-4570-BC85-599C6C120457}" name="Region" dataDxfId="270" dataCellStyle="Neutral"/>
+    <tableColumn id="28" xr3:uid="{6F943A9E-8917-4D9E-B9E7-F4A05FFB81D2}" name="Weather" dataDxfId="269" dataCellStyle="Neutral"/>
+    <tableColumn id="23" xr3:uid="{7894930C-23CD-4521-B98E-3B5BF35910A6}" name="Navigation" dataDxfId="268" dataCellStyle="Neutral"/>
+    <tableColumn id="4" xr3:uid="{1DF1C017-7D5C-4049-8DAB-6EFD6982A8D3}" name="Subject" dataDxfId="267"/>
+    <tableColumn id="5" xr3:uid="{5DC19A03-7D17-498B-872C-75D3C0B8FE97}" name="Description2" dataDxfId="266"/>
+    <tableColumn id="12" xr3:uid="{D1D2B78A-7689-453A-BB50-F1E3BA54F82F}" name="Remarks2" dataDxfId="265"/>
+    <tableColumn id="13" xr3:uid="{46A53FFB-D8FC-4762-A453-F18649266844}" name="Dist (nm)2" dataDxfId="264"/>
+    <tableColumn id="1" xr3:uid="{C4E9AC53-131F-4965-A278-C8805116FF72}" name="Time (u)3" dataDxfId="263"/>
+    <tableColumn id="7" xr3:uid="{CEA136EA-E892-418E-9B76-70DF71C227ED}" name="For4" dataDxfId="262"/>
+    <tableColumn id="8" xr3:uid="{E94A949A-C095-4435-BA47-1E19F13C2CD4}" name="Status5" dataDxfId="261"/>
+    <tableColumn id="9" xr3:uid="{A2004532-A635-4B73-95B0-9A57606A659F}" name="Region6" dataDxfId="260"/>
+    <tableColumn id="10" xr3:uid="{376C73C8-27F3-4D13-8CA3-86B26B6BEABA}" name="Weather7" dataDxfId="259"/>
+    <tableColumn id="11" xr3:uid="{796A7359-26E1-48C4-8A7B-F2AF2A8C071A}" name="Navigation8" dataDxfId="258"/>
+    <tableColumn id="20" xr3:uid="{6CEBCB9B-E078-4B16-BDDF-BCE0F9BE3FE0}" name="original order" dataDxfId="257"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F79926B3-2202-4AD4-A64A-9702EC6DCCA3}" name="Table13" displayName="Table13" ref="A1:AC18" totalsRowShown="0" headerRowDxfId="250" dataDxfId="249">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F79926B3-2202-4AD4-A64A-9702EC6DCCA3}" name="Table13" displayName="Table13" ref="A1:AC18" totalsRowShown="0" headerRowDxfId="256" dataDxfId="255">
   <autoFilter ref="A1:AC18" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AC18">
     <sortCondition ref="G1:G18"/>
   </sortState>
   <tableColumns count="29">
-    <tableColumn id="2" xr3:uid="{A883C4E1-8B3B-4B8A-8613-52FACFFDBCB4}" name="Date" dataDxfId="248" dataCellStyle="Neutral"/>
-    <tableColumn id="3" xr3:uid="{B3112805-4950-44F9-8E8A-AAADDF6D12A3}" name="Hour" dataDxfId="247" dataCellStyle="Neutral"/>
-    <tableColumn id="32" xr3:uid="{5B8D703C-DBFA-426B-AF38-FAD7A800F0DB}" name="Actor" dataDxfId="246" dataCellStyle="Neutral"/>
-    <tableColumn id="22" xr3:uid="{6CC5ED81-D746-43DE-8ECB-EA2AE552241E}" name="eventDefinitionId" dataDxfId="245" dataCellStyle="Neutral"/>
-    <tableColumn id="21" xr3:uid="{ACCD1A6F-5CA7-45B7-9DE8-361019EB0B01}" name="Program" dataDxfId="244" dataCellStyle="Neutral"/>
-    <tableColumn id="6" xr3:uid="{68BBBD50-7FC0-43BC-B969-47236C3D7597}" name="Tool" dataDxfId="243" dataCellStyle="Neutral"/>
-    <tableColumn id="15" xr3:uid="{53875BE8-6DFE-4E1D-A5BD-CEAC49C72D72}" name="Process" dataDxfId="242" dataCellStyle="Neutral"/>
-    <tableColumn id="14" xr3:uid="{76304550-AA3A-4E3D-9817-260F7737FE32}" name="Action" dataDxfId="241" dataCellStyle="Neutral"/>
-    <tableColumn id="16" xr3:uid="{53F8B7EC-C142-452B-AB5B-4121EBD9292A}" name="Label" dataDxfId="240" dataCellStyle="Neutral"/>
-    <tableColumn id="18" xr3:uid="{9DD63867-7B3B-458D-B57B-93DD0826ED30}" name="Station" dataDxfId="239" dataCellStyle="Neutral"/>
-    <tableColumn id="17" xr3:uid="{0D039B87-7EB5-4EF1-BC8C-BE2CE17C4A59}" name="Description" dataDxfId="238" dataCellStyle="Neutral"/>
-    <tableColumn id="31" xr3:uid="{B601E7E0-5E21-4624-A325-D4766B81D0D9}" name="Remarks" dataDxfId="237" dataCellStyle="Neutral"/>
-    <tableColumn id="27" xr3:uid="{B329E4C7-CD4B-4F87-8D41-500531688781}" name="Dist" dataDxfId="236" dataCellStyle="Neutral"/>
-    <tableColumn id="26" xr3:uid="{8C148003-86EF-40CC-A689-0AA3E06DD886}" name="Time" dataDxfId="235" dataCellStyle="Neutral"/>
-    <tableColumn id="24" xr3:uid="{D780F508-B15C-4476-864C-95C2F6539F74}" name="Status" dataDxfId="234" dataCellStyle="Neutral"/>
-    <tableColumn id="29" xr3:uid="{349FBE77-7FC7-43E2-B426-7F0976209284}" name="Region" dataDxfId="233" dataCellStyle="Neutral"/>
-    <tableColumn id="28" xr3:uid="{362703D7-E347-46E4-AD54-7F9C67E96758}" name="Weather" dataDxfId="232" dataCellStyle="Neutral"/>
-    <tableColumn id="23" xr3:uid="{D23C8FBC-D540-4BBA-99FF-D2BADF57CACC}" name="Navigation" dataDxfId="231" dataCellStyle="Neutral"/>
-    <tableColumn id="4" xr3:uid="{044ED456-57AF-4B5C-B1EC-5830CF72E601}" name="Subject" dataDxfId="230"/>
-    <tableColumn id="5" xr3:uid="{BAC2087E-84C9-4DBA-9B56-B0A163C7F58F}" name="Description2" dataDxfId="229"/>
-    <tableColumn id="12" xr3:uid="{7A25CE5A-A0C0-40C9-AB60-1FB2D97E942D}" name="Remarks2" dataDxfId="228"/>
-    <tableColumn id="13" xr3:uid="{4D127608-E09A-4518-81D1-3A80FF3F41E0}" name="Dist (nm)2" dataDxfId="227"/>
-    <tableColumn id="1" xr3:uid="{BE12DED8-825E-4FB7-8580-1C31B68E4901}" name="Time (u)3" dataDxfId="226"/>
-    <tableColumn id="7" xr3:uid="{B6B4D763-C54B-4550-8A13-DEE8873A98FC}" name="For4" dataDxfId="225"/>
-    <tableColumn id="8" xr3:uid="{9C9F7BD0-0ED2-4DF5-B2A9-E22ED38C354C}" name="Status5" dataDxfId="224"/>
-    <tableColumn id="9" xr3:uid="{74BA0754-0093-4197-BAFE-2EBCB909E702}" name="Region6" dataDxfId="223"/>
-    <tableColumn id="10" xr3:uid="{224FFCDE-9EAA-4811-B77E-966560D921AC}" name="Weather7" dataDxfId="222"/>
-    <tableColumn id="11" xr3:uid="{A31F6733-6550-471A-863C-1B97B3A1E1AF}" name="Navigation8" dataDxfId="221"/>
-    <tableColumn id="20" xr3:uid="{77D3E5C0-0CCF-4DB0-9F9B-9D65C7E6A9EC}" name="original order" dataDxfId="220"/>
+    <tableColumn id="2" xr3:uid="{A883C4E1-8B3B-4B8A-8613-52FACFFDBCB4}" name="Date" dataDxfId="254" dataCellStyle="Neutral"/>
+    <tableColumn id="3" xr3:uid="{B3112805-4950-44F9-8E8A-AAADDF6D12A3}" name="Hour" dataDxfId="253" dataCellStyle="Neutral"/>
+    <tableColumn id="32" xr3:uid="{5B8D703C-DBFA-426B-AF38-FAD7A800F0DB}" name="Actor" dataDxfId="252" dataCellStyle="Neutral"/>
+    <tableColumn id="22" xr3:uid="{6CC5ED81-D746-43DE-8ECB-EA2AE552241E}" name="eventDefinitionId" dataDxfId="251" dataCellStyle="Neutral"/>
+    <tableColumn id="21" xr3:uid="{ACCD1A6F-5CA7-45B7-9DE8-361019EB0B01}" name="Program" dataDxfId="250" dataCellStyle="Neutral"/>
+    <tableColumn id="6" xr3:uid="{68BBBD50-7FC0-43BC-B969-47236C3D7597}" name="Tool" dataDxfId="249" dataCellStyle="Neutral"/>
+    <tableColumn id="15" xr3:uid="{53875BE8-6DFE-4E1D-A5BD-CEAC49C72D72}" name="Process" dataDxfId="248" dataCellStyle="Neutral"/>
+    <tableColumn id="14" xr3:uid="{76304550-AA3A-4E3D-9817-260F7737FE32}" name="Action" dataDxfId="247" dataCellStyle="Neutral"/>
+    <tableColumn id="16" xr3:uid="{53F8B7EC-C142-452B-AB5B-4121EBD9292A}" name="Label" dataDxfId="246" dataCellStyle="Neutral"/>
+    <tableColumn id="18" xr3:uid="{9DD63867-7B3B-458D-B57B-93DD0826ED30}" name="Station" dataDxfId="245" dataCellStyle="Neutral"/>
+    <tableColumn id="17" xr3:uid="{0D039B87-7EB5-4EF1-BC8C-BE2CE17C4A59}" name="Description" dataDxfId="244" dataCellStyle="Neutral"/>
+    <tableColumn id="31" xr3:uid="{B601E7E0-5E21-4624-A325-D4766B81D0D9}" name="Remarks" dataDxfId="243" dataCellStyle="Neutral"/>
+    <tableColumn id="27" xr3:uid="{B329E4C7-CD4B-4F87-8D41-500531688781}" name="Dist" dataDxfId="242" dataCellStyle="Neutral"/>
+    <tableColumn id="26" xr3:uid="{8C148003-86EF-40CC-A689-0AA3E06DD886}" name="Time" dataDxfId="241" dataCellStyle="Neutral"/>
+    <tableColumn id="24" xr3:uid="{D780F508-B15C-4476-864C-95C2F6539F74}" name="Status" dataDxfId="240" dataCellStyle="Neutral"/>
+    <tableColumn id="29" xr3:uid="{349FBE77-7FC7-43E2-B426-7F0976209284}" name="Region" dataDxfId="239" dataCellStyle="Neutral"/>
+    <tableColumn id="28" xr3:uid="{362703D7-E347-46E4-AD54-7F9C67E96758}" name="Weather" dataDxfId="238" dataCellStyle="Neutral"/>
+    <tableColumn id="23" xr3:uid="{D23C8FBC-D540-4BBA-99FF-D2BADF57CACC}" name="Navigation" dataDxfId="237" dataCellStyle="Neutral"/>
+    <tableColumn id="4" xr3:uid="{044ED456-57AF-4B5C-B1EC-5830CF72E601}" name="Subject" dataDxfId="236"/>
+    <tableColumn id="5" xr3:uid="{BAC2087E-84C9-4DBA-9B56-B0A163C7F58F}" name="Description2" dataDxfId="235"/>
+    <tableColumn id="12" xr3:uid="{7A25CE5A-A0C0-40C9-AB60-1FB2D97E942D}" name="Remarks2" dataDxfId="234"/>
+    <tableColumn id="13" xr3:uid="{4D127608-E09A-4518-81D1-3A80FF3F41E0}" name="Dist (nm)2" dataDxfId="233"/>
+    <tableColumn id="1" xr3:uid="{BE12DED8-825E-4FB7-8580-1C31B68E4901}" name="Time (u)3" dataDxfId="232"/>
+    <tableColumn id="7" xr3:uid="{B6B4D763-C54B-4550-8A13-DEE8873A98FC}" name="For4" dataDxfId="231"/>
+    <tableColumn id="8" xr3:uid="{9C9F7BD0-0ED2-4DF5-B2A9-E22ED38C354C}" name="Status5" dataDxfId="230"/>
+    <tableColumn id="9" xr3:uid="{74BA0754-0093-4197-BAFE-2EBCB909E702}" name="Region6" dataDxfId="229"/>
+    <tableColumn id="10" xr3:uid="{224FFCDE-9EAA-4811-B77E-966560D921AC}" name="Weather7" dataDxfId="228"/>
+    <tableColumn id="11" xr3:uid="{A31F6733-6550-471A-863C-1B97B3A1E1AF}" name="Navigation8" dataDxfId="227"/>
+    <tableColumn id="20" xr3:uid="{77D3E5C0-0CCF-4DB0-9F9B-9D65C7E6A9EC}" name="original order" dataDxfId="226"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -10022,400 +10082,400 @@
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="K1:K21 K32:K48 K88:K125 K127 K133:K148 L137 K155:K156 K158:K161">
-    <cfRule type="cellIs" dxfId="219" priority="1190" operator="equal">
+    <cfRule type="cellIs" dxfId="225" priority="1190" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1:K53">
-    <cfRule type="cellIs" dxfId="218" priority="199" operator="equal">
+    <cfRule type="cellIs" dxfId="224" priority="201" operator="equal">
+      <formula>"No Impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="223" priority="199" operator="equal">
       <formula>"Interruption"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="217" priority="201" operator="equal">
-      <formula>"No Impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K22:K31">
-    <cfRule type="cellIs" dxfId="216" priority="218" operator="equal">
+    <cfRule type="cellIs" dxfId="222" priority="218" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36">
-    <cfRule type="cellIs" dxfId="215" priority="242" operator="equal">
+    <cfRule type="cellIs" dxfId="221" priority="242" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K49:K52">
-    <cfRule type="cellIs" dxfId="214" priority="212" operator="equal">
+    <cfRule type="cellIs" dxfId="220" priority="212" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K52">
-    <cfRule type="cellIs" dxfId="213" priority="202" operator="equal">
-      <formula>"Heavy impact"</formula>
+    <cfRule type="cellIs" dxfId="219" priority="204" operator="equal">
+      <formula>"No impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="212" priority="203" operator="equal">
+    <cfRule type="cellIs" dxfId="218" priority="203" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="211" priority="204" operator="equal">
-      <formula>"No impact"</formula>
+    <cfRule type="cellIs" dxfId="217" priority="202" operator="equal">
+      <formula>"Heavy impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K53">
-    <cfRule type="cellIs" dxfId="210" priority="200" operator="equal">
+    <cfRule type="cellIs" dxfId="216" priority="200" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K61:K77">
-    <cfRule type="cellIs" dxfId="209" priority="41" operator="equal">
+    <cfRule type="cellIs" dxfId="215" priority="41" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K61:K148 L137">
-    <cfRule type="cellIs" dxfId="208" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="214" priority="4" operator="equal">
       <formula>"Interruption"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="207" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="213" priority="6" operator="equal">
       <formula>"No Impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K78:K87">
-    <cfRule type="cellIs" dxfId="206" priority="83" operator="equal">
+    <cfRule type="cellIs" dxfId="212" priority="83" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K86:K87">
-    <cfRule type="cellIs" dxfId="205" priority="73" operator="equal">
+    <cfRule type="cellIs" dxfId="211" priority="75" operator="equal">
+      <formula>"No impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="210" priority="73" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="204" priority="74" operator="equal">
+    <cfRule type="cellIs" dxfId="209" priority="74" operator="equal">
       <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="203" priority="75" operator="equal">
-      <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K126:K128">
-    <cfRule type="cellIs" dxfId="202" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="208" priority="11" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K129:K134">
-    <cfRule type="cellIs" dxfId="201" priority="23" operator="equal">
+    <cfRule type="cellIs" dxfId="207" priority="23" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K136:K139 L137">
-    <cfRule type="cellIs" dxfId="200" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="206" priority="5" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K155:K156 K158:K161">
-    <cfRule type="cellIs" dxfId="199" priority="1189" operator="equal">
+    <cfRule type="cellIs" dxfId="205" priority="1191" operator="equal">
+      <formula>"No Impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="204" priority="1189" operator="equal">
       <formula>"Interruption"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="198" priority="1191" operator="equal">
-      <formula>"No Impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K167:K173">
-    <cfRule type="cellIs" dxfId="197" priority="925" operator="equal">
-      <formula>"Interruption"</formula>
+    <cfRule type="cellIs" dxfId="203" priority="927" operator="equal">
+      <formula>"No Impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="196" priority="926" operator="equal">
+    <cfRule type="cellIs" dxfId="202" priority="926" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="195" priority="927" operator="equal">
-      <formula>"No Impact"</formula>
+    <cfRule type="cellIs" dxfId="201" priority="925" operator="equal">
+      <formula>"Interruption"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K174">
-    <cfRule type="cellIs" dxfId="194" priority="1144" operator="equal">
+    <cfRule type="cellIs" dxfId="200" priority="1144" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="193" priority="1145" operator="equal">
+    <cfRule type="cellIs" dxfId="199" priority="1145" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="192" priority="1146" operator="equal">
+    <cfRule type="cellIs" dxfId="198" priority="1146" operator="equal">
       <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K175:K182">
-    <cfRule type="cellIs" dxfId="191" priority="913" operator="equal">
-      <formula>"Interruption"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="190" priority="914" operator="equal">
+    <cfRule type="cellIs" dxfId="197" priority="914" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="189" priority="915" operator="equal">
+    <cfRule type="cellIs" dxfId="196" priority="915" operator="equal">
       <formula>"No Impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="195" priority="913" operator="equal">
+      <formula>"Interruption"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K183">
-    <cfRule type="cellIs" dxfId="188" priority="1138" operator="equal">
-      <formula>"Heavy impact"</formula>
+    <cfRule type="cellIs" dxfId="194" priority="1140" operator="equal">
+      <formula>"No impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="187" priority="1139" operator="equal">
+    <cfRule type="cellIs" dxfId="193" priority="1139" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="186" priority="1140" operator="equal">
-      <formula>"No impact"</formula>
+    <cfRule type="cellIs" dxfId="192" priority="1138" operator="equal">
+      <formula>"Heavy impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K184:K193">
-    <cfRule type="cellIs" dxfId="185" priority="895" operator="equal">
+    <cfRule type="cellIs" dxfId="191" priority="896" operator="equal">
+      <formula>"Possible impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="190" priority="895" operator="equal">
       <formula>"Interruption"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="184" priority="896" operator="equal">
-      <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="183" priority="897" operator="equal">
+    <cfRule type="cellIs" dxfId="189" priority="897" operator="equal">
       <formula>"No Impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K194">
-    <cfRule type="cellIs" dxfId="182" priority="1024" operator="equal">
+    <cfRule type="cellIs" dxfId="188" priority="1025" operator="equal">
+      <formula>"Possible impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="187" priority="1024" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="181" priority="1025" operator="equal">
-      <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="180" priority="1026" operator="equal">
+    <cfRule type="cellIs" dxfId="186" priority="1026" operator="equal">
       <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K195:K201">
-    <cfRule type="cellIs" dxfId="179" priority="847" operator="equal">
+    <cfRule type="cellIs" dxfId="185" priority="848" operator="equal">
+      <formula>"Possible impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="184" priority="847" operator="equal">
       <formula>"Interruption"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="178" priority="848" operator="equal">
-      <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="177" priority="849" operator="equal">
+    <cfRule type="cellIs" dxfId="183" priority="849" operator="equal">
       <formula>"No Impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K202:K203">
-    <cfRule type="cellIs" dxfId="176" priority="1000" operator="equal">
+    <cfRule type="cellIs" dxfId="182" priority="1002" operator="equal">
+      <formula>"No impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="181" priority="1000" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="175" priority="1001" operator="equal">
+    <cfRule type="cellIs" dxfId="180" priority="1001" operator="equal">
       <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="174" priority="1002" operator="equal">
-      <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K204:K210">
-    <cfRule type="cellIs" dxfId="173" priority="841" operator="equal">
-      <formula>"Interruption"</formula>
+    <cfRule type="cellIs" dxfId="179" priority="843" operator="equal">
+      <formula>"No Impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="172" priority="842" operator="equal">
+    <cfRule type="cellIs" dxfId="178" priority="842" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="171" priority="843" operator="equal">
-      <formula>"No Impact"</formula>
+    <cfRule type="cellIs" dxfId="177" priority="841" operator="equal">
+      <formula>"Interruption"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K211">
-    <cfRule type="cellIs" dxfId="170" priority="1126" operator="equal">
+    <cfRule type="cellIs" dxfId="176" priority="1128" operator="equal">
+      <formula>"No impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="175" priority="1126" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="169" priority="1127" operator="equal">
+    <cfRule type="cellIs" dxfId="174" priority="1127" operator="equal">
       <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="168" priority="1128" operator="equal">
-      <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K212:K217 K236:K1048576">
-    <cfRule type="cellIs" dxfId="167" priority="1387" operator="equal">
+    <cfRule type="cellIs" dxfId="173" priority="1389" operator="equal">
+      <formula>"No Impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="172" priority="1387" operator="equal">
       <formula>"Interruption"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="166" priority="1388" operator="equal">
+    <cfRule type="cellIs" dxfId="171" priority="1388" operator="equal">
       <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="165" priority="1389" operator="equal">
-      <formula>"No Impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K218">
-    <cfRule type="cellIs" dxfId="164" priority="1120" operator="equal">
+    <cfRule type="cellIs" dxfId="170" priority="1120" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="163" priority="1121" operator="equal">
+    <cfRule type="cellIs" dxfId="169" priority="1121" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="162" priority="1122" operator="equal">
+    <cfRule type="cellIs" dxfId="168" priority="1122" operator="equal">
       <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K219:K235">
-    <cfRule type="cellIs" dxfId="161" priority="829" operator="equal">
+    <cfRule type="cellIs" dxfId="167" priority="830" operator="equal">
+      <formula>"Possible impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="166" priority="829" operator="equal">
       <formula>"Interruption"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="160" priority="830" operator="equal">
-      <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="159" priority="831" operator="equal">
+    <cfRule type="cellIs" dxfId="165" priority="831" operator="equal">
       <formula>"No Impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K18:L18 K88:L113 K114:K118 L116 L119 K120:K125 L121:L125 K155:K156 K158:L161 L167:L235">
-    <cfRule type="cellIs" dxfId="158" priority="1150" operator="equal">
+    <cfRule type="cellIs" dxfId="164" priority="1152" operator="equal">
+      <formula>"No impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="163" priority="1150" operator="equal">
       <formula>"Heavy impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="157" priority="1152" operator="equal">
-      <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K32:L48 K133:L154 K127:L127 K18:L18 K88:L113 K114:K118 L116 L119 K120:K125 L121:L125 K155:K156 K158:L161 L167:L235">
-    <cfRule type="cellIs" dxfId="156" priority="1151" operator="equal">
+    <cfRule type="cellIs" dxfId="162" priority="1151" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K32:L52">
-    <cfRule type="cellIs" dxfId="155" priority="208" operator="equal">
+    <cfRule type="cellIs" dxfId="161" priority="210" operator="equal">
+      <formula>"No impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="160" priority="208" operator="equal">
       <formula>"Heavy impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="154" priority="210" operator="equal">
-      <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K36:L36">
-    <cfRule type="cellIs" dxfId="153" priority="239" operator="equal">
+    <cfRule type="cellIs" dxfId="159" priority="239" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K49:L52">
-    <cfRule type="cellIs" dxfId="152" priority="209" operator="equal">
+    <cfRule type="cellIs" dxfId="158" priority="209" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K54:L85">
-    <cfRule type="cellIs" dxfId="151" priority="37" operator="equal">
-      <formula>"Heavy impact"</formula>
+    <cfRule type="cellIs" dxfId="157" priority="39" operator="equal">
+      <formula>"No impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="150" priority="38" operator="equal">
+    <cfRule type="cellIs" dxfId="156" priority="38" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="149" priority="39" operator="equal">
-      <formula>"No impact"</formula>
+    <cfRule type="cellIs" dxfId="155" priority="37" operator="equal">
+      <formula>"Heavy impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K126:L127">
-    <cfRule type="cellIs" dxfId="148" priority="7" operator="equal">
-      <formula>"Heavy impact"</formula>
+    <cfRule type="cellIs" dxfId="154" priority="9" operator="equal">
+      <formula>"No impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="147" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="153" priority="8" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="146" priority="9" operator="equal">
-      <formula>"No impact"</formula>
+    <cfRule type="cellIs" dxfId="152" priority="7" operator="equal">
+      <formula>"Heavy impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K129:L134">
-    <cfRule type="cellIs" dxfId="145" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="151" priority="20" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K129:L154">
-    <cfRule type="cellIs" dxfId="144" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="150" priority="3" operator="equal">
+      <formula>"No impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="149" priority="1" operator="equal">
       <formula>"Heavy impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="143" priority="3" operator="equal">
-      <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K136:L139">
-    <cfRule type="cellIs" dxfId="142" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="148" priority="2" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K166:L166">
-    <cfRule type="cellIs" dxfId="141" priority="262" operator="equal">
-      <formula>"Heavy impact"</formula>
+    <cfRule type="cellIs" dxfId="147" priority="264" operator="equal">
+      <formula>"No impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="140" priority="263" operator="equal">
+    <cfRule type="cellIs" dxfId="146" priority="263" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="139" priority="264" operator="equal">
-      <formula>"No impact"</formula>
+    <cfRule type="cellIs" dxfId="145" priority="262" operator="equal">
+      <formula>"Heavy impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L1:L31">
-    <cfRule type="cellIs" dxfId="138" priority="214" operator="equal">
-      <formula>"Heavy impact"</formula>
+    <cfRule type="cellIs" dxfId="144" priority="216" operator="equal">
+      <formula>"No impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="137" priority="215" operator="equal">
+    <cfRule type="cellIs" dxfId="143" priority="215" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="136" priority="216" operator="equal">
-      <formula>"No impact"</formula>
+    <cfRule type="cellIs" dxfId="142" priority="214" operator="equal">
+      <formula>"Heavy impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L52:L53">
-    <cfRule type="cellIs" dxfId="135" priority="196" operator="equal">
-      <formula>"Heavy impact"</formula>
+    <cfRule type="cellIs" dxfId="141" priority="198" operator="equal">
+      <formula>"No impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="134" priority="197" operator="equal">
+    <cfRule type="cellIs" dxfId="140" priority="197" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="133" priority="198" operator="equal">
-      <formula>"No impact"</formula>
+    <cfRule type="cellIs" dxfId="139" priority="196" operator="equal">
+      <formula>"Heavy impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L86:L87">
-    <cfRule type="cellIs" dxfId="132" priority="76" operator="equal">
-      <formula>"Heavy impact"</formula>
+    <cfRule type="cellIs" dxfId="138" priority="78" operator="equal">
+      <formula>"No impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="131" priority="77" operator="equal">
+    <cfRule type="cellIs" dxfId="137" priority="77" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="130" priority="78" operator="equal">
-      <formula>"No impact"</formula>
+    <cfRule type="cellIs" dxfId="136" priority="76" operator="equal">
+      <formula>"Heavy impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L128">
-    <cfRule type="cellIs" dxfId="129" priority="25" operator="equal">
-      <formula>"Heavy impact"</formula>
+    <cfRule type="cellIs" dxfId="135" priority="27" operator="equal">
+      <formula>"No impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="128" priority="26" operator="equal">
+    <cfRule type="cellIs" dxfId="134" priority="26" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="127" priority="27" operator="equal">
-      <formula>"No impact"</formula>
+    <cfRule type="cellIs" dxfId="133" priority="25" operator="equal">
+      <formula>"Heavy impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L138:L139">
-    <cfRule type="cellIs" dxfId="126" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="132" priority="13" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="125" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="131" priority="15" operator="equal">
+      <formula>"No impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="130" priority="14" operator="equal">
       <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="124" priority="15" operator="equal">
-      <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L155:L156">
-    <cfRule type="cellIs" dxfId="123" priority="259" operator="equal">
+    <cfRule type="cellIs" dxfId="129" priority="259" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="122" priority="260" operator="equal">
+    <cfRule type="cellIs" dxfId="128" priority="261" operator="equal">
+      <formula>"No impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="127" priority="260" operator="equal">
       <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="121" priority="261" operator="equal">
-      <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L236:L1048576">
-    <cfRule type="cellIs" dxfId="120" priority="1384" operator="equal">
+    <cfRule type="cellIs" dxfId="126" priority="1384" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="119" priority="1385" operator="equal">
+    <cfRule type="cellIs" dxfId="125" priority="1385" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="118" priority="1386" operator="equal">
+    <cfRule type="cellIs" dxfId="124" priority="1386" operator="equal">
       <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -21951,405 +22011,405 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F1:AC3 B2:E2">
-    <cfRule type="notContainsBlanks" dxfId="117" priority="1">
+    <cfRule type="notContainsBlanks" dxfId="123" priority="1">
       <formula>LEN(TRIM(B1))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA5:AA26 AA37:AA53 AA93:AA130 AA132 AA138:AA153 AB142 AA160:AA161 AA163:AA166">
-    <cfRule type="cellIs" dxfId="116" priority="96" operator="equal">
+    <cfRule type="cellIs" dxfId="122" priority="96" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA5:AA58">
-    <cfRule type="cellIs" dxfId="115" priority="34" operator="equal">
+    <cfRule type="cellIs" dxfId="121" priority="36" operator="equal">
+      <formula>"No Impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="120" priority="34" operator="equal">
       <formula>"Interruption"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="114" priority="36" operator="equal">
-      <formula>"No Impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA27:AA36">
-    <cfRule type="cellIs" dxfId="113" priority="47" operator="equal">
+    <cfRule type="cellIs" dxfId="119" priority="47" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA41">
-    <cfRule type="cellIs" dxfId="112" priority="49" operator="equal">
+    <cfRule type="cellIs" dxfId="118" priority="49" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA54:AA57">
-    <cfRule type="cellIs" dxfId="111" priority="43" operator="equal">
+    <cfRule type="cellIs" dxfId="117" priority="43" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA57">
-    <cfRule type="cellIs" dxfId="110" priority="37" operator="equal">
+    <cfRule type="cellIs" dxfId="116" priority="39" operator="equal">
+      <formula>"No impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="115" priority="37" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="109" priority="38" operator="equal">
+    <cfRule type="cellIs" dxfId="114" priority="38" operator="equal">
       <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="108" priority="39" operator="equal">
-      <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA58">
-    <cfRule type="cellIs" dxfId="107" priority="35" operator="equal">
+    <cfRule type="cellIs" dxfId="113" priority="35" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA66:AA82">
-    <cfRule type="cellIs" dxfId="106" priority="23" operator="equal">
+    <cfRule type="cellIs" dxfId="112" priority="23" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA66:AA153 AB142">
-    <cfRule type="cellIs" dxfId="105" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="111" priority="5" operator="equal">
       <formula>"Interruption"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="104" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="110" priority="7" operator="equal">
       <formula>"No Impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA83:AA92">
-    <cfRule type="cellIs" dxfId="103" priority="30" operator="equal">
+    <cfRule type="cellIs" dxfId="109" priority="30" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA91:AA92">
-    <cfRule type="cellIs" dxfId="102" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="108" priority="25" operator="equal">
+      <formula>"Possible impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="107" priority="24" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="101" priority="25" operator="equal">
-      <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="100" priority="26" operator="equal">
+    <cfRule type="cellIs" dxfId="106" priority="26" operator="equal">
       <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA131:AA133">
-    <cfRule type="cellIs" dxfId="99" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="105" priority="11" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA134:AA139">
-    <cfRule type="cellIs" dxfId="98" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="104" priority="16" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA141:AA144 AB142">
-    <cfRule type="cellIs" dxfId="97" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="103" priority="6" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA160:AA161 AA163:AA166">
-    <cfRule type="cellIs" dxfId="96" priority="95" operator="equal">
+    <cfRule type="cellIs" dxfId="102" priority="95" operator="equal">
       <formula>"Interruption"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="95" priority="97" operator="equal">
+    <cfRule type="cellIs" dxfId="101" priority="97" operator="equal">
       <formula>"No Impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA172:AA178">
-    <cfRule type="cellIs" dxfId="94" priority="71" operator="equal">
-      <formula>"Interruption"</formula>
+    <cfRule type="cellIs" dxfId="100" priority="73" operator="equal">
+      <formula>"No Impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="93" priority="72" operator="equal">
+    <cfRule type="cellIs" dxfId="99" priority="72" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="92" priority="73" operator="equal">
-      <formula>"No Impact"</formula>
+    <cfRule type="cellIs" dxfId="98" priority="71" operator="equal">
+      <formula>"Interruption"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA179">
-    <cfRule type="cellIs" dxfId="91" priority="89" operator="equal">
+    <cfRule type="cellIs" dxfId="97" priority="90" operator="equal">
+      <formula>"Possible impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="96" priority="89" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="90" priority="90" operator="equal">
-      <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="89" priority="91" operator="equal">
+    <cfRule type="cellIs" dxfId="95" priority="91" operator="equal">
       <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA180:AA187">
-    <cfRule type="cellIs" dxfId="88" priority="68" operator="equal">
-      <formula>"Interruption"</formula>
+    <cfRule type="cellIs" dxfId="94" priority="70" operator="equal">
+      <formula>"No Impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="87" priority="69" operator="equal">
+    <cfRule type="cellIs" dxfId="93" priority="69" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="86" priority="70" operator="equal">
-      <formula>"No Impact"</formula>
+    <cfRule type="cellIs" dxfId="92" priority="68" operator="equal">
+      <formula>"Interruption"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA188">
-    <cfRule type="cellIs" dxfId="85" priority="86" operator="equal">
-      <formula>"Heavy impact"</formula>
+    <cfRule type="cellIs" dxfId="91" priority="88" operator="equal">
+      <formula>"No impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="84" priority="87" operator="equal">
+    <cfRule type="cellIs" dxfId="90" priority="87" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="83" priority="88" operator="equal">
-      <formula>"No impact"</formula>
+    <cfRule type="cellIs" dxfId="89" priority="86" operator="equal">
+      <formula>"Heavy impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA189:AA198">
-    <cfRule type="cellIs" dxfId="82" priority="65" operator="equal">
-      <formula>"Interruption"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="81" priority="66" operator="equal">
+    <cfRule type="cellIs" dxfId="88" priority="66" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="80" priority="67" operator="equal">
+    <cfRule type="cellIs" dxfId="87" priority="67" operator="equal">
       <formula>"No Impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="86" priority="65" operator="equal">
+      <formula>"Interruption"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA199">
-    <cfRule type="cellIs" dxfId="79" priority="77" operator="equal">
-      <formula>"Heavy impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="78" priority="78" operator="equal">
+    <cfRule type="cellIs" dxfId="85" priority="78" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="77" priority="79" operator="equal">
+    <cfRule type="cellIs" dxfId="84" priority="79" operator="equal">
       <formula>"No impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="83" priority="77" operator="equal">
+      <formula>"Heavy impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA200:AA206">
-    <cfRule type="cellIs" dxfId="76" priority="62" operator="equal">
+    <cfRule type="cellIs" dxfId="82" priority="62" operator="equal">
       <formula>"Interruption"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="75" priority="63" operator="equal">
+    <cfRule type="cellIs" dxfId="81" priority="63" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="74" priority="64" operator="equal">
+    <cfRule type="cellIs" dxfId="80" priority="64" operator="equal">
       <formula>"No Impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA207:AA208">
-    <cfRule type="cellIs" dxfId="73" priority="74" operator="equal">
+    <cfRule type="cellIs" dxfId="79" priority="74" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="72" priority="75" operator="equal">
+    <cfRule type="cellIs" dxfId="78" priority="76" operator="equal">
+      <formula>"No impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="77" priority="75" operator="equal">
       <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="71" priority="76" operator="equal">
-      <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA209:AA215">
-    <cfRule type="cellIs" dxfId="70" priority="59" operator="equal">
+    <cfRule type="cellIs" dxfId="76" priority="59" operator="equal">
       <formula>"Interruption"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="69" priority="60" operator="equal">
+    <cfRule type="cellIs" dxfId="75" priority="60" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="68" priority="61" operator="equal">
+    <cfRule type="cellIs" dxfId="74" priority="61" operator="equal">
       <formula>"No Impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA216">
-    <cfRule type="cellIs" dxfId="67" priority="83" operator="equal">
-      <formula>"Heavy impact"</formula>
+    <cfRule type="cellIs" dxfId="73" priority="85" operator="equal">
+      <formula>"No impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="66" priority="84" operator="equal">
+    <cfRule type="cellIs" dxfId="72" priority="84" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="65" priority="85" operator="equal">
-      <formula>"No impact"</formula>
+    <cfRule type="cellIs" dxfId="71" priority="83" operator="equal">
+      <formula>"Heavy impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA217:AA222 AA241:AA1048576">
-    <cfRule type="cellIs" dxfId="64" priority="101" operator="equal">
+    <cfRule type="cellIs" dxfId="70" priority="102" operator="equal">
+      <formula>"Possible impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="69" priority="101" operator="equal">
       <formula>"Interruption"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="63" priority="102" operator="equal">
-      <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="62" priority="103" operator="equal">
+    <cfRule type="cellIs" dxfId="68" priority="103" operator="equal">
       <formula>"No Impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA223">
-    <cfRule type="cellIs" dxfId="61" priority="80" operator="equal">
+    <cfRule type="cellIs" dxfId="67" priority="80" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="81" operator="equal">
+    <cfRule type="cellIs" dxfId="66" priority="82" operator="equal">
+      <formula>"No impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="65" priority="81" operator="equal">
       <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="59" priority="82" operator="equal">
-      <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA224:AA240">
-    <cfRule type="cellIs" dxfId="58" priority="56" operator="equal">
+    <cfRule type="cellIs" dxfId="64" priority="56" operator="equal">
       <formula>"Interruption"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="57" priority="57" operator="equal">
+    <cfRule type="cellIs" dxfId="63" priority="57" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="58" operator="equal">
+    <cfRule type="cellIs" dxfId="62" priority="58" operator="equal">
       <formula>"No Impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA23:AB23 AA93:AB118 AA119:AA123 AB121 AB124 AA125:AA130 AB126:AB130 AA160:AA161 AA163:AB166 AB172:AB240">
-    <cfRule type="cellIs" dxfId="55" priority="92" operator="equal">
+    <cfRule type="cellIs" dxfId="61" priority="94" operator="equal">
+      <formula>"No impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="60" priority="92" operator="equal">
       <formula>"Heavy impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="94" operator="equal">
-      <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA37:AB53 AA138:AB159 AA132:AB132 AA23:AB23 AA93:AB118 AA119:AA123 AB121 AB124 AA125:AA130 AB126:AB130 AA160:AA161 AA163:AB166 AB172:AB240">
-    <cfRule type="cellIs" dxfId="53" priority="93" operator="equal">
+    <cfRule type="cellIs" dxfId="59" priority="93" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA37:AB57">
-    <cfRule type="cellIs" dxfId="52" priority="40" operator="equal">
+    <cfRule type="cellIs" dxfId="58" priority="42" operator="equal">
+      <formula>"No impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="57" priority="40" operator="equal">
       <formula>"Heavy impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="42" operator="equal">
-      <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA41:AB41">
-    <cfRule type="cellIs" dxfId="50" priority="48" operator="equal">
+    <cfRule type="cellIs" dxfId="56" priority="48" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA54:AB57">
-    <cfRule type="cellIs" dxfId="49" priority="41" operator="equal">
+    <cfRule type="cellIs" dxfId="55" priority="41" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA59:AB90">
-    <cfRule type="cellIs" dxfId="48" priority="20" operator="equal">
-      <formula>"Heavy impact"</formula>
+    <cfRule type="cellIs" dxfId="54" priority="22" operator="equal">
+      <formula>"No impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="47" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="53" priority="21" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="22" operator="equal">
-      <formula>"No impact"</formula>
+    <cfRule type="cellIs" dxfId="52" priority="20" operator="equal">
+      <formula>"Heavy impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA131:AB132">
-    <cfRule type="cellIs" dxfId="45" priority="8" operator="equal">
-      <formula>"Heavy impact"</formula>
+    <cfRule type="cellIs" dxfId="51" priority="10" operator="equal">
+      <formula>"No impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="50" priority="9" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="10" operator="equal">
-      <formula>"No impact"</formula>
+    <cfRule type="cellIs" dxfId="49" priority="8" operator="equal">
+      <formula>"Heavy impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA134:AB139">
-    <cfRule type="cellIs" dxfId="42" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="48" priority="15" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA134:AB159">
-    <cfRule type="cellIs" dxfId="41" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="47" priority="4" operator="equal">
+      <formula>"No impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="46" priority="2" operator="equal">
       <formula>"Heavy impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="4" operator="equal">
-      <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA141:AB144">
-    <cfRule type="cellIs" dxfId="39" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="45" priority="3" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA171:AB171">
-    <cfRule type="cellIs" dxfId="38" priority="53" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="53" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="54" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="54" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="55" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="55" operator="equal">
       <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB5:AB36">
-    <cfRule type="cellIs" dxfId="35" priority="44" operator="equal">
-      <formula>"Heavy impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="45" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="45" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="46" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="46" operator="equal">
       <formula>"No impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="39" priority="44" operator="equal">
+      <formula>"Heavy impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB57:AB58">
-    <cfRule type="cellIs" dxfId="32" priority="31" operator="equal">
-      <formula>"Heavy impact"</formula>
+    <cfRule type="cellIs" dxfId="38" priority="33" operator="equal">
+      <formula>"No impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="32" operator="equal">
+    <cfRule type="cellIs" dxfId="37" priority="32" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="33" operator="equal">
-      <formula>"No impact"</formula>
+    <cfRule type="cellIs" dxfId="36" priority="31" operator="equal">
+      <formula>"Heavy impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB91:AB92">
-    <cfRule type="cellIs" dxfId="29" priority="27" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="29" operator="equal">
+      <formula>"No impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="34" priority="27" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="28" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="28" operator="equal">
       <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="29" operator="equal">
-      <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB133">
-    <cfRule type="cellIs" dxfId="26" priority="17" operator="equal">
-      <formula>"Heavy impact"</formula>
+    <cfRule type="cellIs" dxfId="32" priority="19" operator="equal">
+      <formula>"No impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="18" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="19" operator="equal">
-      <formula>"No impact"</formula>
+    <cfRule type="cellIs" dxfId="30" priority="17" operator="equal">
+      <formula>"Heavy impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB143:AB144">
-    <cfRule type="cellIs" dxfId="23" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="14" operator="equal">
+      <formula>"No impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="28" priority="12" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="13" operator="equal">
       <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="14" operator="equal">
-      <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB160:AB161">
-    <cfRule type="cellIs" dxfId="20" priority="50" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="50" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="51" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="51" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="52" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="52" operator="equal">
       <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB241:AB1048576">
-    <cfRule type="cellIs" dxfId="17" priority="98" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="98" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="99" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="99" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="100" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="100" operator="equal">
       <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -22408,7 +22468,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC18"/>
+  <dimension ref="A1:AC19"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="15" style="32" customWidth="1"/>
@@ -23495,64 +23555,126 @@
         <v>18</v>
       </c>
     </row>
+    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A19" s="33"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="43"/>
+      <c r="E19" s="43"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="36"/>
+      <c r="H19" s="36"/>
+      <c r="I19" s="58" t="s">
+        <v>66</v>
+      </c>
+      <c r="J19" s="58" t="s">
+        <v>95</v>
+      </c>
+      <c r="K19" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="L19" s="58"/>
+      <c r="M19" s="58"/>
+      <c r="N19" s="58"/>
+      <c r="O19" s="58"/>
+      <c r="P19" s="58"/>
+      <c r="Q19" s="58"/>
+      <c r="R19" s="58"/>
+      <c r="S19" s="47" t="s">
+        <v>66</v>
+      </c>
+      <c r="T19" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="U19" s="22" t="s">
+        <v>107</v>
+      </c>
+      <c r="V19" s="47"/>
+      <c r="W19" s="47"/>
+      <c r="X19" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y19" s="47" t="s">
+        <v>10</v>
+      </c>
+      <c r="Z19" s="47" t="s">
+        <v>85</v>
+      </c>
+      <c r="AA19" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB19" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="AC19" s="22">
+        <v>18</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
-  <conditionalFormatting sqref="AA1:AA18">
-    <cfRule type="cellIs" dxfId="14" priority="104" operator="equal">
+  <conditionalFormatting sqref="AA1:AA19">
+    <cfRule type="cellIs" dxfId="8" priority="45" operator="equal">
+      <formula>"Interruption"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="47" operator="equal">
+      <formula>"No Impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="107" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA1:AA18">
-    <cfRule type="cellIs" dxfId="13" priority="42" operator="equal">
+  <conditionalFormatting sqref="AA20:AA1048576">
+    <cfRule type="cellIs" dxfId="20" priority="82" operator="equal">
       <formula>"Interruption"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="44" operator="equal">
-      <formula>"No Impact"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AB19:AB1048576">
-    <cfRule type="cellIs" dxfId="11" priority="45" operator="equal">
-      <formula>"Heavy impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="46" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="83" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="47" operator="equal">
-      <formula>"No impact"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AA19:AA1048576">
-    <cfRule type="cellIs" dxfId="8" priority="79" operator="equal">
-      <formula>"Interruption"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="80" operator="equal">
-      <formula>"Possible impact"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="81" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="84" operator="equal">
       <formula>"No Impact"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA12:AB18">
-    <cfRule type="cellIs" dxfId="5" priority="100" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="103" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="102" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="104" operator="equal">
+      <formula>"Possible impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="15" priority="105" operator="equal">
       <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA12:AB18">
-    <cfRule type="cellIs" dxfId="3" priority="101" operator="equal">
+  <conditionalFormatting sqref="AB1:AB11">
+    <cfRule type="cellIs" dxfId="14" priority="55" operator="equal">
+      <formula>"Heavy impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="13" priority="56" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="57" operator="equal">
+      <formula>"No impact"</formula>
+    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB1:AB11">
-    <cfRule type="cellIs" dxfId="2" priority="52" operator="equal">
+  <conditionalFormatting sqref="AB20:AB1048576">
+    <cfRule type="cellIs" dxfId="11" priority="48" operator="equal">
       <formula>"Heavy impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="53" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="49" operator="equal">
       <formula>"Possible impact"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="54" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="50" operator="equal">
+      <formula>"No impact"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA19:AB19">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+      <formula>"Heavy impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>"Possible impact"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
       <formula>"No impact"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -23574,13 +23696,13 @@
           <x14:formula1>
             <xm:f>List!$D$2:$D$5</xm:f>
           </x14:formula1>
-          <xm:sqref>X19:X1048576 X3:X12</xm:sqref>
+          <xm:sqref>X3:X12 X20:X1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2D61B9B7-47BC-4776-BF3E-7E4BAD45D92A}">
           <x14:formula1>
             <xm:f>List!$F$2:$F$7</xm:f>
           </x14:formula1>
-          <xm:sqref>AB3:AB11 AB19:AB1048576 AA12:AB18</xm:sqref>
+          <xm:sqref>AB3:AB11 AA12:AB19 AB20:AB1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D0E8E517-F102-440E-82D2-9F4168164A52}">
           <x14:formula1>

</xml_diff>